<commit_message>
Working code on S3 mini Mic interface
</commit_message>
<xml_diff>
--- a/IOT Based FireAlarm Detector.xlsx
+++ b/IOT Based FireAlarm Detector.xlsx
@@ -5,11 +5,11 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP i7\OneDrive\Desktop\FireAlarm Detection and Alert System\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FireAlarm Detection and Alert System\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="7470" windowHeight="2805" tabRatio="683"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="7476" windowHeight="2808" tabRatio="683"/>
   </bookViews>
   <sheets>
     <sheet name="Plant Monitoring Sensor Network" sheetId="12" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="148">
   <si>
     <t>Project Dashboard - Comprehensive Project Tracking System</t>
   </si>
@@ -509,6 +509,18 @@
   </si>
   <si>
     <t>Hanna Latif-Walmsley</t>
+  </si>
+  <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>In Process</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Waiting For the Components </t>
+  </si>
+  <si>
+    <t>Next Phase (Planned Soon)</t>
   </si>
 </sst>
 </file>
@@ -1224,7 +1236,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="225">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1429,9 +1441,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1521,50 +1530,83 @@
     <xf numFmtId="49" fontId="9" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="9" fillId="5" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1575,65 +1617,102 @@
     <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="15" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1648,177 +1727,107 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="15" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="5" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2105,13 +2114,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>42</xdr:row>
-          <xdr:rowOff>219075</xdr:rowOff>
+          <xdr:rowOff>220980</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>66675</xdr:colOff>
+          <xdr:colOff>68580</xdr:colOff>
           <xdr:row>44</xdr:row>
           <xdr:rowOff>38100</xdr:rowOff>
         </xdr:to>
@@ -2169,13 +2178,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>43</xdr:row>
-          <xdr:rowOff>142875</xdr:rowOff>
+          <xdr:rowOff>144780</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>45</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2233,15 +2242,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>45</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>66675</xdr:colOff>
+          <xdr:colOff>68580</xdr:colOff>
           <xdr:row>47</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2297,13 +2306,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>46</xdr:row>
           <xdr:rowOff>152400</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>48</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2361,15 +2370,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>47</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>49</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2425,15 +2434,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>48</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>50</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2489,15 +2498,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>49</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>51</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2555,11 +2564,11 @@
           <xdr:col>1</xdr:col>
           <xdr:colOff>533400</xdr:colOff>
           <xdr:row>50</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>160020</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>52</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2617,13 +2626,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>51</xdr:row>
           <xdr:rowOff>152400</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>53</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2681,13 +2690,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>523875</xdr:colOff>
+          <xdr:colOff>525780</xdr:colOff>
           <xdr:row>44</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>160020</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>66675</xdr:colOff>
+          <xdr:colOff>68580</xdr:colOff>
           <xdr:row>46</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2745,13 +2754,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>809625</xdr:colOff>
+          <xdr:colOff>807720</xdr:colOff>
           <xdr:row>7</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>971550</xdr:colOff>
+          <xdr:colOff>975360</xdr:colOff>
           <xdr:row>8</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -2809,15 +2818,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>857250</xdr:colOff>
+          <xdr:colOff>861060</xdr:colOff>
           <xdr:row>6</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>2</xdr:col>
-          <xdr:colOff>1552575</xdr:colOff>
+          <xdr:colOff>1554480</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>9525</xdr:rowOff>
+          <xdr:rowOff>7620</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -2873,15 +2882,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>57150</xdr:colOff>
+          <xdr:colOff>60960</xdr:colOff>
           <xdr:row>8</xdr:row>
-          <xdr:rowOff>171450</xdr:rowOff>
+          <xdr:rowOff>175260</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>1</xdr:col>
-          <xdr:colOff>219075</xdr:colOff>
+          <xdr:colOff>220980</xdr:colOff>
           <xdr:row>9</xdr:row>
-          <xdr:rowOff>161925</xdr:rowOff>
+          <xdr:rowOff>160020</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -3423,96 +3432,96 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G103"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="37.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="17" style="1" customWidth="1"/>
-    <col min="3" max="3" width="45.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="3" max="3" width="45.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="28.77734375" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="128" t="s">
+    <row r="1" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="198" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="129"/>
-      <c r="C1" s="129"/>
-      <c r="D1" s="129"/>
-      <c r="E1" s="129"/>
-      <c r="F1" s="130"/>
-    </row>
-    <row r="2" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="131" t="s">
+      <c r="B1" s="199"/>
+      <c r="C1" s="199"/>
+      <c r="D1" s="199"/>
+      <c r="E1" s="199"/>
+      <c r="F1" s="200"/>
+    </row>
+    <row r="2" spans="1:6" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="201" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="132"/>
-      <c r="C2" s="132"/>
-      <c r="D2" s="132"/>
-      <c r="E2" s="132"/>
-      <c r="F2" s="133"/>
-    </row>
-    <row r="3" spans="1:6" ht="4.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="131"/>
-      <c r="B3" s="132"/>
-      <c r="C3" s="132"/>
-      <c r="D3" s="132"/>
-      <c r="E3" s="132"/>
-      <c r="F3" s="133"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B2" s="202"/>
+      <c r="C2" s="202"/>
+      <c r="D2" s="202"/>
+      <c r="E2" s="202"/>
+      <c r="F2" s="203"/>
+    </row>
+    <row r="3" spans="1:6" ht="4.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="201"/>
+      <c r="B3" s="202"/>
+      <c r="C3" s="202"/>
+      <c r="D3" s="202"/>
+      <c r="E3" s="202"/>
+      <c r="F3" s="203"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="134"/>
-      <c r="C4" s="135"/>
-      <c r="D4" s="135"/>
-      <c r="E4" s="135"/>
-      <c r="F4" s="136"/>
-    </row>
-    <row r="5" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B4" s="144"/>
+      <c r="C4" s="145"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="145"/>
+      <c r="F4" s="146"/>
+    </row>
+    <row r="5" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="58" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="137" t="s">
+      <c r="B5" s="204" t="s">
         <v>142</v>
       </c>
-      <c r="C5" s="137"/>
-      <c r="D5" s="137"/>
-      <c r="E5" s="137"/>
-      <c r="F5" s="138"/>
-    </row>
-    <row r="6" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C5" s="204"/>
+      <c r="D5" s="204"/>
+      <c r="E5" s="204"/>
+      <c r="F5" s="205"/>
+    </row>
+    <row r="6" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A6" s="59" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="139" t="s">
+      <c r="B6" s="206" t="s">
         <v>143</v>
       </c>
-      <c r="C6" s="139"/>
-      <c r="D6" s="139"/>
-      <c r="E6" s="139"/>
-      <c r="F6" s="140"/>
-    </row>
-    <row r="7" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C6" s="206"/>
+      <c r="D6" s="206"/>
+      <c r="E6" s="206"/>
+      <c r="F6" s="207"/>
+    </row>
+    <row r="7" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A7" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="141">
+      <c r="B7" s="208">
         <v>45969</v>
       </c>
-      <c r="C7" s="142"/>
+      <c r="C7" s="209"/>
       <c r="D7" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="141" t="s">
+      <c r="E7" s="208" t="s">
         <v>131</v>
       </c>
-      <c r="F7" s="143"/>
-    </row>
-    <row r="8" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="F7" s="210"/>
+    </row>
+    <row r="8" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
         <v>7</v>
       </c>
@@ -3522,26 +3531,26 @@
       <c r="C8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="144"/>
-      <c r="F8" s="145"/>
-    </row>
-    <row r="9" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E8" s="211"/>
+      <c r="F8" s="212"/>
+    </row>
+    <row r="9" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A9" s="59" t="s">
         <v>10</v>
       </c>
-      <c r="B9" s="146">
+      <c r="B9" s="213">
         <v>21</v>
       </c>
-      <c r="C9" s="146"/>
-      <c r="D9" s="147" t="s">
+      <c r="C9" s="213"/>
+      <c r="D9" s="214" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="147"/>
+      <c r="E9" s="214"/>
       <c r="F9" s="15" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A10" s="59" t="s">
         <v>12</v>
       </c>
@@ -3551,92 +3560,92 @@
       <c r="E10" s="62"/>
       <c r="F10" s="63"/>
     </row>
-    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A11" s="148"/>
-      <c r="B11" s="149"/>
-      <c r="C11" s="149"/>
-      <c r="D11" s="149"/>
-      <c r="E11" s="149"/>
-      <c r="F11" s="150"/>
+    <row r="11" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A11" s="215"/>
+      <c r="B11" s="216"/>
+      <c r="C11" s="216"/>
+      <c r="D11" s="216"/>
+      <c r="E11" s="216"/>
+      <c r="F11" s="217"/>
     </row>
     <row r="12" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="151" t="s">
+      <c r="A12" s="218" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="152"/>
-      <c r="C12" s="152"/>
-      <c r="D12" s="152"/>
-      <c r="E12" s="152"/>
-      <c r="F12" s="153"/>
-    </row>
-    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="119"/>
-      <c r="B13" s="120"/>
-      <c r="C13" s="120"/>
-      <c r="D13" s="120"/>
-      <c r="E13" s="120"/>
-      <c r="F13" s="121"/>
-    </row>
-    <row r="14" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="122"/>
-      <c r="B14" s="123"/>
-      <c r="C14" s="123"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="123"/>
-      <c r="F14" s="124"/>
-    </row>
-    <row r="15" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="122"/>
-      <c r="B15" s="123"/>
-      <c r="C15" s="123"/>
-      <c r="D15" s="123"/>
-      <c r="E15" s="123"/>
-      <c r="F15" s="124"/>
-    </row>
-    <row r="16" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="122"/>
-      <c r="B16" s="123"/>
-      <c r="C16" s="123"/>
-      <c r="D16" s="123"/>
-      <c r="E16" s="123"/>
-      <c r="F16" s="124"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="122"/>
-      <c r="B17" s="123"/>
-      <c r="C17" s="123"/>
-      <c r="D17" s="123"/>
-      <c r="E17" s="123"/>
-      <c r="F17" s="124"/>
-    </row>
-    <row r="18" spans="1:6" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="125"/>
-      <c r="B18" s="126"/>
-      <c r="C18" s="126"/>
-      <c r="D18" s="126"/>
-      <c r="E18" s="126"/>
-      <c r="F18" s="127"/>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B12" s="219"/>
+      <c r="C12" s="219"/>
+      <c r="D12" s="219"/>
+      <c r="E12" s="219"/>
+      <c r="F12" s="220"/>
+    </row>
+    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="189"/>
+      <c r="B13" s="190"/>
+      <c r="C13" s="190"/>
+      <c r="D13" s="190"/>
+      <c r="E13" s="190"/>
+      <c r="F13" s="191"/>
+    </row>
+    <row r="14" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="192"/>
+      <c r="B14" s="193"/>
+      <c r="C14" s="193"/>
+      <c r="D14" s="193"/>
+      <c r="E14" s="193"/>
+      <c r="F14" s="194"/>
+    </row>
+    <row r="15" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="192"/>
+      <c r="B15" s="193"/>
+      <c r="C15" s="193"/>
+      <c r="D15" s="193"/>
+      <c r="E15" s="193"/>
+      <c r="F15" s="194"/>
+    </row>
+    <row r="16" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="192"/>
+      <c r="B16" s="193"/>
+      <c r="C16" s="193"/>
+      <c r="D16" s="193"/>
+      <c r="E16" s="193"/>
+      <c r="F16" s="194"/>
+    </row>
+    <row r="17" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="192"/>
+      <c r="B17" s="193"/>
+      <c r="C17" s="193"/>
+      <c r="D17" s="193"/>
+      <c r="E17" s="193"/>
+      <c r="F17" s="194"/>
+    </row>
+    <row r="18" spans="1:6" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="195"/>
+      <c r="B18" s="196"/>
+      <c r="C18" s="196"/>
+      <c r="D18" s="196"/>
+      <c r="E18" s="196"/>
+      <c r="F18" s="197"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="64" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="154" t="s">
+      <c r="B19" s="143" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="155"/>
+      <c r="C19" s="187"/>
       <c r="D19" s="65"/>
-      <c r="E19" s="155"/>
-      <c r="F19" s="156"/>
-    </row>
-    <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A20" s="192" t="s">
+      <c r="E19" s="187"/>
+      <c r="F19" s="188"/>
+    </row>
+    <row r="20" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A20" s="118" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="157" t="s">
+      <c r="B20" s="180" t="s">
         <v>16</v>
       </c>
-      <c r="C20" s="158"/>
+      <c r="C20" s="181"/>
       <c r="D20" s="66" t="s">
         <v>115</v>
       </c>
@@ -3647,89 +3656,113 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="193"/>
-      <c r="B21" s="159" t="s">
+    <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="119"/>
+      <c r="B21" s="182" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="160"/>
-      <c r="D21" s="69"/>
-      <c r="E21" s="161" t="s">
+      <c r="C21" s="183"/>
+      <c r="D21" s="69">
+        <v>4</v>
+      </c>
+      <c r="E21" s="184" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="70"/>
-    </row>
-    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A22" s="193"/>
-      <c r="B22" s="164" t="s">
+      <c r="F21" s="70" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A22" s="119"/>
+      <c r="B22" s="121" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="165"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="162"/>
-      <c r="F22" s="70"/>
-    </row>
-    <row r="23" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="193"/>
-      <c r="B23" s="164" t="s">
+      <c r="C22" s="122"/>
+      <c r="D22" s="71">
+        <v>9</v>
+      </c>
+      <c r="E22" s="185"/>
+      <c r="F22" s="70" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A23" s="119"/>
+      <c r="B23" s="121" t="s">
         <v>100</v>
       </c>
-      <c r="C23" s="165"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="162"/>
-      <c r="F23" s="72"/>
-    </row>
-    <row r="24" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A24" s="193"/>
-      <c r="B24" s="164" t="s">
+      <c r="C23" s="122"/>
+      <c r="D23" s="71">
+        <v>3</v>
+      </c>
+      <c r="E23" s="185"/>
+      <c r="F23" s="70" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A24" s="119"/>
+      <c r="B24" s="121" t="s">
         <v>98</v>
       </c>
-      <c r="C24" s="165"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="162"/>
-      <c r="F24" s="72"/>
-    </row>
-    <row r="25" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="193"/>
-      <c r="B25" s="164" t="s">
+      <c r="C24" s="122"/>
+      <c r="D24" s="71">
+        <v>22</v>
+      </c>
+      <c r="E24" s="185"/>
+      <c r="F24" s="70" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A25" s="119"/>
+      <c r="B25" s="121" t="s">
         <v>101</v>
       </c>
-      <c r="C25" s="165"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="162"/>
-      <c r="F25" s="72"/>
-    </row>
-    <row r="26" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="194"/>
-      <c r="B26" s="164" t="s">
+      <c r="C25" s="122"/>
+      <c r="D25" s="71">
+        <v>8</v>
+      </c>
+      <c r="E25" s="185"/>
+      <c r="F25" s="70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A26" s="120"/>
+      <c r="B26" s="121" t="s">
         <v>133</v>
       </c>
-      <c r="C26" s="165"/>
-      <c r="D26" s="73"/>
-      <c r="E26" s="162"/>
-      <c r="F26" s="72"/>
-    </row>
-    <row r="27" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C26" s="122"/>
+      <c r="D26" s="72">
+        <v>0</v>
+      </c>
+      <c r="E26" s="185"/>
+      <c r="F26" s="70" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
-      <c r="B27" s="166" t="s">
+      <c r="B27" s="137" t="s">
         <v>116</v>
       </c>
-      <c r="C27" s="167"/>
-      <c r="D27" s="74">
+      <c r="C27" s="138"/>
+      <c r="D27" s="73">
         <f>SUM(D21:D26)</f>
-        <v>0</v>
-      </c>
-      <c r="E27" s="163"/>
-      <c r="F27" s="75"/>
-    </row>
-    <row r="28" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A28" s="168" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="186"/>
+      <c r="F27" s="74"/>
+    </row>
+    <row r="28" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A28" s="179" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="157" t="s">
+      <c r="B28" s="180" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="158"/>
+      <c r="C28" s="181"/>
       <c r="D28" s="66" t="s">
         <v>115</v>
       </c>
@@ -3740,77 +3773,91 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="168"/>
-      <c r="B29" s="164" t="s">
+    <row r="29" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A29" s="179"/>
+      <c r="B29" s="121" t="s">
         <v>134</v>
       </c>
-      <c r="C29" s="165"/>
-      <c r="D29" s="69"/>
-      <c r="E29" s="161" t="s">
+      <c r="C29" s="122"/>
+      <c r="D29" s="69">
+        <v>5</v>
+      </c>
+      <c r="E29" s="184" t="s">
         <v>136</v>
       </c>
-      <c r="F29" s="70"/>
-    </row>
-    <row r="30" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A30" s="168"/>
-      <c r="B30" s="164" t="s">
+      <c r="F29" s="70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A30" s="179"/>
+      <c r="B30" s="121" t="s">
         <v>135</v>
       </c>
-      <c r="C30" s="165"/>
-      <c r="D30" s="71"/>
-      <c r="E30" s="162"/>
-      <c r="F30" s="72"/>
-    </row>
-    <row r="31" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A31" s="168"/>
-      <c r="B31" s="164" t="s">
+      <c r="C30" s="122"/>
+      <c r="D30" s="71">
+        <v>4</v>
+      </c>
+      <c r="E30" s="185"/>
+      <c r="F30" s="70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A31" s="179"/>
+      <c r="B31" s="121" t="s">
         <v>102</v>
       </c>
-      <c r="C31" s="165"/>
-      <c r="D31" s="71"/>
-      <c r="E31" s="162"/>
-      <c r="F31" s="72"/>
-    </row>
-    <row r="32" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A32" s="168"/>
-      <c r="B32" s="164" t="s">
+      <c r="C31" s="122"/>
+      <c r="D31" s="71">
+        <v>7</v>
+      </c>
+      <c r="E31" s="185"/>
+      <c r="F31" s="70" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A32" s="179"/>
+      <c r="B32" s="121" t="s">
         <v>103</v>
       </c>
-      <c r="C32" s="165"/>
+      <c r="C32" s="122"/>
       <c r="D32" s="71"/>
-      <c r="E32" s="162"/>
-      <c r="F32" s="72"/>
-    </row>
-    <row r="33" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A33" s="168"/>
-      <c r="B33" s="159"/>
-      <c r="C33" s="160"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="162"/>
-      <c r="F33" s="72"/>
-    </row>
-    <row r="34" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E32" s="185"/>
+      <c r="F32" s="70" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A33" s="179"/>
+      <c r="B33" s="182"/>
+      <c r="C33" s="183"/>
+      <c r="D33" s="72"/>
+      <c r="E33" s="185"/>
+      <c r="F33" s="70"/>
+    </row>
+    <row r="34" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A34" s="25"/>
-      <c r="B34" s="166" t="s">
+      <c r="B34" s="137" t="s">
         <v>117</v>
       </c>
-      <c r="C34" s="167"/>
-      <c r="D34" s="74">
+      <c r="C34" s="138"/>
+      <c r="D34" s="73">
         <f>SUM(D29:D33)</f>
-        <v>0</v>
-      </c>
-      <c r="E34" s="163"/>
-      <c r="F34" s="75"/>
-    </row>
-    <row r="35" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A35" s="168" t="s">
+        <v>16</v>
+      </c>
+      <c r="E34" s="186"/>
+      <c r="F34" s="74"/>
+    </row>
+    <row r="35" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A35" s="179" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="157" t="s">
+      <c r="B35" s="180" t="s">
         <v>16</v>
       </c>
-      <c r="C35" s="158"/>
+      <c r="C35" s="181"/>
       <c r="D35" s="66" t="s">
         <v>115</v>
       </c>
@@ -3821,291 +3868,301 @@
         <v>18</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A36" s="168"/>
-      <c r="B36" s="159" t="s">
+    <row r="36" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A36" s="179"/>
+      <c r="B36" s="182" t="s">
         <v>104</v>
       </c>
-      <c r="C36" s="160"/>
+      <c r="C36" s="183"/>
       <c r="D36" s="69"/>
-      <c r="E36" s="161" t="s">
+      <c r="E36" s="184" t="s">
         <v>108</v>
       </c>
-      <c r="F36" s="70"/>
-    </row>
-    <row r="37" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A37" s="168"/>
-      <c r="B37" s="159" t="s">
+      <c r="F36" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A37" s="179"/>
+      <c r="B37" s="182" t="s">
         <v>137</v>
       </c>
-      <c r="C37" s="160"/>
+      <c r="C37" s="183"/>
       <c r="D37" s="71"/>
-      <c r="E37" s="162"/>
-      <c r="F37" s="72"/>
-    </row>
-    <row r="38" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A38" s="168"/>
-      <c r="B38" s="159" t="s">
+      <c r="E37" s="185"/>
+      <c r="F37" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A38" s="179"/>
+      <c r="B38" s="182" t="s">
         <v>105</v>
       </c>
-      <c r="C38" s="160"/>
+      <c r="C38" s="183"/>
       <c r="D38" s="71"/>
-      <c r="E38" s="162"/>
-      <c r="F38" s="72"/>
-    </row>
-    <row r="39" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A39" s="168"/>
-      <c r="B39" s="159" t="s">
+      <c r="E38" s="185"/>
+      <c r="F38" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A39" s="179"/>
+      <c r="B39" s="182" t="s">
         <v>99</v>
       </c>
-      <c r="C39" s="160"/>
+      <c r="C39" s="183"/>
       <c r="D39" s="71"/>
-      <c r="E39" s="162"/>
-      <c r="F39" s="72"/>
-    </row>
-    <row r="40" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A40" s="168"/>
-      <c r="B40" s="159" t="s">
+      <c r="E39" s="185"/>
+      <c r="F39" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A40" s="179"/>
+      <c r="B40" s="182" t="s">
         <v>106</v>
       </c>
-      <c r="C40" s="160"/>
-      <c r="D40" s="73"/>
-      <c r="E40" s="162"/>
-      <c r="F40" s="72"/>
-    </row>
-    <row r="41" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="C40" s="183"/>
+      <c r="D40" s="72"/>
+      <c r="E40" s="185"/>
+      <c r="F40" s="70" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A41" s="25"/>
-      <c r="B41" s="166" t="s">
+      <c r="B41" s="137" t="s">
         <v>118</v>
       </c>
-      <c r="C41" s="167"/>
-      <c r="D41" s="74">
+      <c r="C41" s="138"/>
+      <c r="D41" s="73">
         <f>SUM(D36:D40)</f>
         <v>0</v>
       </c>
       <c r="E41" s="24"/>
-      <c r="F41" s="76"/>
-    </row>
-    <row r="42" spans="1:6" s="2" customFormat="1" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A42" s="209"/>
-      <c r="B42" s="210"/>
-      <c r="C42" s="210"/>
-      <c r="D42" s="210"/>
-      <c r="E42" s="210"/>
-      <c r="F42" s="211"/>
+      <c r="F41" s="75"/>
+    </row>
+    <row r="42" spans="1:6" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A42" s="139"/>
+      <c r="B42" s="140"/>
+      <c r="C42" s="140"/>
+      <c r="D42" s="140"/>
+      <c r="E42" s="140"/>
+      <c r="F42" s="141"/>
     </row>
     <row r="43" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="212" t="s">
+      <c r="A43" s="142" t="s">
         <v>21</v>
       </c>
-      <c r="B43" s="154"/>
-      <c r="C43" s="77" t="s">
+      <c r="B43" s="143"/>
+      <c r="C43" s="76" t="s">
         <v>22</v>
       </c>
-      <c r="D43" s="134" t="s">
+      <c r="D43" s="144" t="s">
         <v>23</v>
       </c>
-      <c r="E43" s="135"/>
-      <c r="F43" s="136"/>
-    </row>
-    <row r="44" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E43" s="145"/>
+      <c r="F43" s="146"/>
+    </row>
+    <row r="44" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A44" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="78"/>
+      <c r="B44" s="77"/>
       <c r="C44" s="55" t="s">
         <v>25</v>
       </c>
-      <c r="D44" s="213" t="s">
+      <c r="D44" s="147" t="s">
         <v>26</v>
       </c>
-      <c r="E44" s="214"/>
-      <c r="F44" s="215"/>
-    </row>
-    <row r="45" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E44" s="148"/>
+      <c r="F44" s="149"/>
+    </row>
+    <row r="45" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A45" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B45" s="78"/>
+      <c r="B45" s="77"/>
       <c r="C45" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="D45" s="216"/>
-      <c r="E45" s="217"/>
-      <c r="F45" s="218"/>
-    </row>
-    <row r="46" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="D45" s="150"/>
+      <c r="E45" s="151"/>
+      <c r="F45" s="152"/>
+    </row>
+    <row r="46" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A46" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="B46" s="78"/>
+      <c r="B46" s="77"/>
       <c r="C46" s="54" t="s">
         <v>114</v>
       </c>
-      <c r="D46" s="216"/>
-      <c r="E46" s="217"/>
-      <c r="F46" s="218"/>
-    </row>
-    <row r="47" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="D46" s="150"/>
+      <c r="E46" s="151"/>
+      <c r="F46" s="152"/>
+    </row>
+    <row r="47" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A47" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="B47" s="78"/>
+      <c r="B47" s="77"/>
       <c r="C47" s="54" t="s">
         <v>30</v>
       </c>
-      <c r="D47" s="216"/>
-      <c r="E47" s="217"/>
-      <c r="F47" s="218"/>
-    </row>
-    <row r="48" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="D47" s="150"/>
+      <c r="E47" s="151"/>
+      <c r="F47" s="152"/>
+    </row>
+    <row r="48" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A48" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B48" s="78"/>
+      <c r="B48" s="77"/>
       <c r="C48" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="D48" s="219"/>
-      <c r="E48" s="220"/>
-      <c r="F48" s="221"/>
-    </row>
-    <row r="49" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="D48" s="153"/>
+      <c r="E48" s="154"/>
+      <c r="F48" s="155"/>
+    </row>
+    <row r="49" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A49" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B49" s="78"/>
+      <c r="B49" s="77"/>
       <c r="C49" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D49" s="169" t="s">
+      <c r="D49" s="176" t="s">
         <v>34</v>
       </c>
-      <c r="E49" s="170"/>
-      <c r="F49" s="171"/>
-    </row>
-    <row r="50" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E49" s="177"/>
+      <c r="F49" s="178"/>
+    </row>
+    <row r="50" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A50" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B50" s="78"/>
+      <c r="B50" s="77"/>
       <c r="C50" s="56" t="s">
         <v>113</v>
       </c>
-      <c r="D50" s="201" t="s">
+      <c r="D50" s="129" t="s">
         <v>109</v>
       </c>
-      <c r="E50" s="202"/>
-      <c r="F50" s="203"/>
-    </row>
-    <row r="51" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E50" s="130"/>
+      <c r="F50" s="131"/>
+    </row>
+    <row r="51" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="B51" s="78"/>
+      <c r="B51" s="77"/>
       <c r="C51" s="56" t="s">
         <v>140</v>
       </c>
-      <c r="D51" s="201" t="s">
+      <c r="D51" s="129" t="s">
         <v>112</v>
       </c>
-      <c r="E51" s="202"/>
-      <c r="F51" s="203"/>
-    </row>
-    <row r="52" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E51" s="130"/>
+      <c r="F51" s="131"/>
+    </row>
+    <row r="52" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A52" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B52" s="78"/>
+      <c r="B52" s="77"/>
       <c r="C52" s="56" t="s">
         <v>111</v>
       </c>
-      <c r="D52" s="201" t="s">
+      <c r="D52" s="129" t="s">
         <v>110</v>
       </c>
-      <c r="E52" s="202"/>
-      <c r="F52" s="203"/>
-    </row>
-    <row r="53" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="E52" s="130"/>
+      <c r="F52" s="131"/>
+    </row>
+    <row r="53" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A53" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B53" s="78"/>
+      <c r="B53" s="77"/>
       <c r="C53" s="56"/>
-      <c r="D53" s="201"/>
-      <c r="E53" s="202"/>
-      <c r="F53" s="203"/>
-    </row>
-    <row r="54" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A54" s="204"/>
-      <c r="B54" s="205"/>
-      <c r="C54" s="205"/>
-      <c r="D54" s="205"/>
-      <c r="E54" s="205"/>
-      <c r="F54" s="206"/>
-    </row>
-    <row r="55" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A55" s="195" t="s">
+      <c r="D53" s="129"/>
+      <c r="E53" s="130"/>
+      <c r="F53" s="131"/>
+    </row>
+    <row r="54" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A54" s="132"/>
+      <c r="B54" s="133"/>
+      <c r="C54" s="133"/>
+      <c r="D54" s="133"/>
+      <c r="E54" s="133"/>
+      <c r="F54" s="134"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="123" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="207"/>
-      <c r="C55" s="207"/>
-      <c r="D55" s="207"/>
-      <c r="E55" s="207"/>
-      <c r="F55" s="208"/>
-    </row>
-    <row r="56" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A56" s="181" t="s">
+      <c r="B55" s="135"/>
+      <c r="C55" s="135"/>
+      <c r="D55" s="135"/>
+      <c r="E55" s="135"/>
+      <c r="F55" s="136"/>
+    </row>
+    <row r="56" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A56" s="165" t="s">
         <v>120</v>
       </c>
-      <c r="B56" s="181"/>
-      <c r="C56" s="181"/>
-      <c r="D56" s="181"/>
-      <c r="E56" s="181"/>
-      <c r="F56" s="79" t="s">
+      <c r="B56" s="165"/>
+      <c r="C56" s="165"/>
+      <c r="D56" s="165"/>
+      <c r="E56" s="165"/>
+      <c r="F56" s="78" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A57" s="182"/>
-      <c r="B57" s="182"/>
-      <c r="C57" s="182"/>
-      <c r="D57" s="182"/>
-      <c r="E57" s="182"/>
-      <c r="F57" s="80"/>
-    </row>
-    <row r="58" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A58" s="182"/>
-      <c r="B58" s="182"/>
-      <c r="C58" s="182"/>
-      <c r="D58" s="182"/>
-      <c r="E58" s="182"/>
-      <c r="F58" s="81"/>
-    </row>
-    <row r="59" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A59" s="82" t="s">
+    <row r="57" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A57" s="166"/>
+      <c r="B57" s="166"/>
+      <c r="C57" s="166"/>
+      <c r="D57" s="166"/>
+      <c r="E57" s="166"/>
+      <c r="F57" s="79"/>
+    </row>
+    <row r="58" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A58" s="166"/>
+      <c r="B58" s="166"/>
+      <c r="C58" s="166"/>
+      <c r="D58" s="166"/>
+      <c r="E58" s="166"/>
+      <c r="F58" s="80"/>
+    </row>
+    <row r="59" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A59" s="81" t="s">
         <v>141</v>
       </c>
-      <c r="B59" s="83"/>
-      <c r="C59" s="183" t="s">
+      <c r="B59" s="82"/>
+      <c r="C59" s="167" t="s">
         <v>121</v>
       </c>
-      <c r="D59" s="184"/>
-      <c r="E59" s="185"/>
-      <c r="F59" s="84">
+      <c r="D59" s="168"/>
+      <c r="E59" s="169"/>
+      <c r="F59" s="83">
         <f>SUM(F57:F58)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A60" s="186"/>
-      <c r="B60" s="187"/>
-      <c r="C60" s="187"/>
-      <c r="D60" s="187"/>
-      <c r="E60" s="187"/>
-      <c r="F60" s="188"/>
-    </row>
-    <row r="61" spans="1:6" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A60" s="170"/>
+      <c r="B60" s="171"/>
+      <c r="C60" s="171"/>
+      <c r="D60" s="171"/>
+      <c r="E60" s="171"/>
+      <c r="F60" s="172"/>
+    </row>
+    <row r="61" spans="1:6" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="27" t="s">
         <v>122</v>
       </c>
@@ -4115,7 +4172,7 @@
       <c r="E61" s="26"/>
       <c r="F61" s="28"/>
     </row>
-    <row r="62" spans="1:6" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="16" t="s">
         <v>44</v>
       </c>
@@ -4128,14 +4185,14 @@
       <c r="D62" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E62" s="85" t="s">
+      <c r="E62" s="84" t="s">
         <v>48</v>
       </c>
-      <c r="F62" s="86" t="s">
+      <c r="F62" s="85" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A63" s="17" t="s">
         <v>50</v>
       </c>
@@ -4144,13 +4201,13 @@
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="10"/>
-      <c r="E63" s="87"/>
-      <c r="F63" s="88">
+      <c r="E63" s="86"/>
+      <c r="F63" s="87">
         <f>D63*E63</f>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A64" s="17" t="s">
         <v>52</v>
       </c>
@@ -4159,13 +4216,13 @@
       </c>
       <c r="C64" s="9"/>
       <c r="D64" s="10"/>
-      <c r="E64" s="87"/>
-      <c r="F64" s="88">
+      <c r="E64" s="86"/>
+      <c r="F64" s="87">
         <f t="shared" ref="F64:F70" si="0">D64*E64</f>
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A65" s="17" t="s">
         <v>54</v>
       </c>
@@ -4174,13 +4231,13 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="10"/>
-      <c r="E65" s="87"/>
-      <c r="F65" s="88">
+      <c r="E65" s="86"/>
+      <c r="F65" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A66" s="18" t="s">
         <v>56</v>
       </c>
@@ -4189,13 +4246,13 @@
       </c>
       <c r="C66" s="9"/>
       <c r="D66" s="10"/>
-      <c r="E66" s="87"/>
-      <c r="F66" s="88">
+      <c r="E66" s="86"/>
+      <c r="F66" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A67" s="18" t="s">
         <v>58</v>
       </c>
@@ -4204,13 +4261,13 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="10"/>
-      <c r="E67" s="87"/>
-      <c r="F67" s="88">
+      <c r="E67" s="86"/>
+      <c r="F67" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A68" s="18" t="s">
         <v>60</v>
       </c>
@@ -4219,13 +4276,13 @@
       </c>
       <c r="C68" s="9"/>
       <c r="D68" s="10"/>
-      <c r="E68" s="87"/>
-      <c r="F68" s="88">
+      <c r="E68" s="86"/>
+      <c r="F68" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A69" s="17" t="s">
         <v>62</v>
       </c>
@@ -4234,397 +4291,446 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="10"/>
-      <c r="E69" s="87"/>
-      <c r="F69" s="88">
+      <c r="E69" s="86"/>
+      <c r="F69" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A70" s="19" t="s">
         <v>64</v>
       </c>
       <c r="B70" s="11"/>
       <c r="C70" s="12"/>
-      <c r="D70" s="89"/>
-      <c r="E70" s="87"/>
-      <c r="F70" s="88">
+      <c r="D70" s="88"/>
+      <c r="E70" s="86"/>
+      <c r="F70" s="87">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="31"/>
       <c r="B71" s="30"/>
       <c r="C71" s="29"/>
       <c r="D71" s="32"/>
-      <c r="E71" s="90" t="s">
+      <c r="E71" s="89" t="s">
         <v>65</v>
       </c>
-      <c r="F71" s="91">
+      <c r="F71" s="90">
         <f>SUM(F63:F70)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A72" s="189"/>
-      <c r="B72" s="190"/>
-      <c r="C72" s="190"/>
-      <c r="D72" s="190"/>
-      <c r="E72" s="190"/>
-      <c r="F72" s="191"/>
-    </row>
-    <row r="73" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="195" t="s">
+    <row r="72" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A72" s="173"/>
+      <c r="B72" s="174"/>
+      <c r="C72" s="174"/>
+      <c r="D72" s="174"/>
+      <c r="E72" s="174"/>
+      <c r="F72" s="175"/>
+    </row>
+    <row r="73" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="123" t="s">
         <v>123</v>
       </c>
-      <c r="B73" s="196"/>
-      <c r="C73" s="196"/>
-      <c r="D73" s="196"/>
-      <c r="E73" s="196"/>
-      <c r="F73" s="197"/>
-    </row>
-    <row r="74" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="198" t="s">
+      <c r="B73" s="124"/>
+      <c r="C73" s="124"/>
+      <c r="D73" s="124"/>
+      <c r="E73" s="124"/>
+      <c r="F73" s="125"/>
+    </row>
+    <row r="74" spans="1:7" s="3" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="126" t="s">
         <v>124</v>
       </c>
-      <c r="B74" s="199"/>
-      <c r="C74" s="199"/>
-      <c r="D74" s="199"/>
-      <c r="E74" s="199"/>
-      <c r="F74" s="200"/>
-    </row>
-    <row r="75" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A75" s="92" t="s">
+      <c r="B74" s="127"/>
+      <c r="C74" s="127"/>
+      <c r="D74" s="127"/>
+      <c r="E74" s="127"/>
+      <c r="F74" s="128"/>
+    </row>
+    <row r="75" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A75" s="91" t="s">
         <v>39</v>
       </c>
-      <c r="B75" s="93" t="s">
+      <c r="B75" s="92" t="s">
         <v>125</v>
       </c>
-      <c r="C75" s="94" t="s">
+      <c r="C75" s="93" t="s">
         <v>126</v>
       </c>
-      <c r="D75" s="95" t="s">
+      <c r="D75" s="94" t="s">
         <v>127</v>
       </c>
-      <c r="E75" s="96" t="s">
+      <c r="E75" s="95" t="s">
         <v>40</v>
       </c>
-      <c r="F75" s="97" t="s">
+      <c r="F75" s="96" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="76" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A76" s="98" t="s">
+    <row r="76" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A76" s="97" t="s">
         <v>15</v>
       </c>
-      <c r="B76" s="99">
+      <c r="B76" s="98">
         <f>B9</f>
         <v>21</v>
       </c>
-      <c r="C76" s="100">
+      <c r="C76" s="99">
         <f>D27</f>
-        <v>0</v>
-      </c>
-      <c r="D76" s="101">
+        <v>46</v>
+      </c>
+      <c r="D76" s="100">
         <f>B76*C76</f>
-        <v>0</v>
-      </c>
-      <c r="E76" s="102"/>
-      <c r="F76" s="103">
+        <v>966</v>
+      </c>
+      <c r="E76" s="101">
+        <v>500</v>
+      </c>
+      <c r="F76" s="102">
         <f>D76-E76</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A77" s="98" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A77" s="97" t="s">
         <v>19</v>
       </c>
-      <c r="B77" s="99">
+      <c r="B77" s="98">
         <f>B9</f>
         <v>21</v>
       </c>
-      <c r="C77" s="100">
+      <c r="C77" s="99">
         <f>D34</f>
-        <v>0</v>
-      </c>
-      <c r="D77" s="101">
+        <v>16</v>
+      </c>
+      <c r="D77" s="100">
         <f t="shared" ref="D77:D79" si="1">B77*C77</f>
-        <v>0</v>
-      </c>
-      <c r="E77" s="102"/>
-      <c r="F77" s="103">
+        <v>336</v>
+      </c>
+      <c r="E77" s="101"/>
+      <c r="F77" s="102">
         <f t="shared" ref="F77:F80" si="2">D77-E77</f>
-        <v>0</v>
-      </c>
-      <c r="G77" s="104"/>
-    </row>
-    <row r="78" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A78" s="105" t="s">
+        <v>336</v>
+      </c>
+      <c r="G77" s="103"/>
+    </row>
+    <row r="78" spans="1:7" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A78" s="104" t="s">
         <v>20</v>
       </c>
-      <c r="B78" s="106">
+      <c r="B78" s="105">
         <f>B9</f>
         <v>21</v>
       </c>
-      <c r="C78" s="107">
+      <c r="C78" s="106">
         <f>D41</f>
         <v>0</v>
       </c>
-      <c r="D78" s="108">
+      <c r="D78" s="107">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E78" s="109"/>
-      <c r="F78" s="110">
+      <c r="E78" s="108"/>
+      <c r="F78" s="109">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="111" t="s">
+    <row r="79" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="110" t="s">
         <v>128</v>
       </c>
-      <c r="B79" s="112">
+      <c r="B79" s="111">
         <f>B9</f>
         <v>21</v>
       </c>
-      <c r="C79" s="113">
+      <c r="C79" s="112">
         <f>F59</f>
         <v>0</v>
       </c>
-      <c r="D79" s="114">
+      <c r="D79" s="113">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="E79" s="114"/>
-      <c r="F79" s="114">
+      <c r="E79" s="113"/>
+      <c r="F79" s="113">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="111" t="s">
+    <row r="80" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="110" t="s">
         <v>66</v>
       </c>
-      <c r="B80" s="112" t="s">
+      <c r="B80" s="111" t="s">
         <v>129</v>
       </c>
-      <c r="C80" s="113" t="s">
+      <c r="C80" s="112" t="s">
         <v>130</v>
       </c>
-      <c r="D80" s="114">
+      <c r="D80" s="113">
         <f>F71</f>
         <v>0</v>
       </c>
-      <c r="E80" s="114"/>
-      <c r="F80" s="114">
+      <c r="E80" s="113"/>
+      <c r="F80" s="113">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="115" t="s">
+    <row r="81" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="114" t="s">
         <v>42</v>
       </c>
-      <c r="B81" s="115"/>
-      <c r="C81" s="116">
+      <c r="B81" s="114"/>
+      <c r="C81" s="115">
         <f>SUM(C76:C79)</f>
-        <v>0</v>
-      </c>
-      <c r="D81" s="117">
+        <v>62</v>
+      </c>
+      <c r="D81" s="116">
         <f>SUM(D76:D80)</f>
-        <v>0</v>
-      </c>
-      <c r="E81" s="117">
+        <v>1302</v>
+      </c>
+      <c r="E81" s="116">
         <f>SUM(E76:E79)</f>
-        <v>0</v>
-      </c>
-      <c r="F81" s="117">
+        <v>500</v>
+      </c>
+      <c r="F81" s="116">
         <f>SUM(F76:F80)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="118"/>
-      <c r="B82" s="118"/>
-      <c r="C82" s="118"/>
-      <c r="D82" s="118"/>
-      <c r="E82" s="118"/>
-      <c r="F82" s="118"/>
-    </row>
-    <row r="83" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="118"/>
-      <c r="B83" s="118"/>
-      <c r="C83" s="118"/>
-      <c r="D83" s="118"/>
-      <c r="E83" s="118"/>
-      <c r="F83" s="118"/>
-    </row>
-    <row r="84" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="172" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A82" s="117"/>
+      <c r="B82" s="117"/>
+      <c r="C82" s="117"/>
+      <c r="D82" s="117"/>
+      <c r="E82" s="117"/>
+      <c r="F82" s="117"/>
+    </row>
+    <row r="83" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A83" s="117"/>
+      <c r="B83" s="117"/>
+      <c r="C83" s="117"/>
+      <c r="D83" s="117"/>
+      <c r="E83" s="117"/>
+      <c r="F83" s="117"/>
+    </row>
+    <row r="84" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A84" s="156" t="s">
         <v>43</v>
       </c>
-      <c r="B84" s="173"/>
-      <c r="C84" s="173"/>
-      <c r="D84" s="173"/>
-      <c r="E84" s="173"/>
-      <c r="F84" s="174"/>
-    </row>
-    <row r="85" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A85" s="175"/>
-      <c r="B85" s="176"/>
-      <c r="C85" s="176"/>
-      <c r="D85" s="176"/>
-      <c r="E85" s="176"/>
-      <c r="F85" s="177"/>
-    </row>
-    <row r="86" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A86" s="175"/>
-      <c r="B86" s="176"/>
-      <c r="C86" s="176"/>
-      <c r="D86" s="176"/>
-      <c r="E86" s="176"/>
-      <c r="F86" s="177"/>
-    </row>
-    <row r="87" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A87" s="175"/>
-      <c r="B87" s="176"/>
-      <c r="C87" s="176"/>
-      <c r="D87" s="176"/>
-      <c r="E87" s="176"/>
-      <c r="F87" s="177"/>
-    </row>
-    <row r="88" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A88" s="175"/>
-      <c r="B88" s="176"/>
-      <c r="C88" s="176"/>
-      <c r="D88" s="176"/>
-      <c r="E88" s="176"/>
-      <c r="F88" s="177"/>
-    </row>
-    <row r="89" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A89" s="175"/>
-      <c r="B89" s="176"/>
-      <c r="C89" s="176"/>
-      <c r="D89" s="176"/>
-      <c r="E89" s="176"/>
-      <c r="F89" s="177"/>
-    </row>
-    <row r="90" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="175"/>
-      <c r="B90" s="176"/>
-      <c r="C90" s="176"/>
-      <c r="D90" s="176"/>
-      <c r="E90" s="176"/>
-      <c r="F90" s="177"/>
-    </row>
-    <row r="91" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="175"/>
-      <c r="B91" s="176"/>
-      <c r="C91" s="176"/>
-      <c r="D91" s="176"/>
-      <c r="E91" s="176"/>
-      <c r="F91" s="177"/>
-    </row>
-    <row r="92" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="175"/>
-      <c r="B92" s="176"/>
-      <c r="C92" s="176"/>
-      <c r="D92" s="176"/>
-      <c r="E92" s="176"/>
-      <c r="F92" s="177"/>
-    </row>
-    <row r="93" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="175"/>
-      <c r="B93" s="176"/>
-      <c r="C93" s="176"/>
-      <c r="D93" s="176"/>
-      <c r="E93" s="176"/>
-      <c r="F93" s="177"/>
-    </row>
-    <row r="94" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="175"/>
-      <c r="B94" s="176"/>
-      <c r="C94" s="176"/>
-      <c r="D94" s="176"/>
-      <c r="E94" s="176"/>
-      <c r="F94" s="177"/>
-    </row>
-    <row r="95" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="175"/>
-      <c r="B95" s="176"/>
-      <c r="C95" s="176"/>
-      <c r="D95" s="176"/>
-      <c r="E95" s="176"/>
-      <c r="F95" s="177"/>
-    </row>
-    <row r="96" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="175"/>
-      <c r="B96" s="176"/>
-      <c r="C96" s="176"/>
-      <c r="D96" s="176"/>
-      <c r="E96" s="176"/>
-      <c r="F96" s="177"/>
-    </row>
-    <row r="97" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="175"/>
-      <c r="B97" s="176"/>
-      <c r="C97" s="176"/>
-      <c r="D97" s="176"/>
-      <c r="E97" s="176"/>
-      <c r="F97" s="177"/>
-    </row>
-    <row r="98" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="175"/>
-      <c r="B98" s="176"/>
-      <c r="C98" s="176"/>
-      <c r="D98" s="176"/>
-      <c r="E98" s="176"/>
-      <c r="F98" s="177"/>
-    </row>
-    <row r="99" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="175"/>
-      <c r="B99" s="176"/>
-      <c r="C99" s="176"/>
-      <c r="D99" s="176"/>
-      <c r="E99" s="176"/>
-      <c r="F99" s="177"/>
-    </row>
-    <row r="100" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="175"/>
-      <c r="B100" s="176"/>
-      <c r="C100" s="176"/>
-      <c r="D100" s="176"/>
-      <c r="E100" s="176"/>
-      <c r="F100" s="177"/>
-    </row>
-    <row r="101" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="175"/>
-      <c r="B101" s="176"/>
-      <c r="C101" s="176"/>
-      <c r="D101" s="176"/>
-      <c r="E101" s="176"/>
-      <c r="F101" s="177"/>
-    </row>
-    <row r="102" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="175"/>
-      <c r="B102" s="176"/>
-      <c r="C102" s="176"/>
-      <c r="D102" s="176"/>
-      <c r="E102" s="176"/>
-      <c r="F102" s="177"/>
-    </row>
-    <row r="103" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="178"/>
-      <c r="B103" s="179"/>
-      <c r="C103" s="179"/>
-      <c r="D103" s="179"/>
-      <c r="E103" s="179"/>
-      <c r="F103" s="180"/>
+      <c r="B84" s="157"/>
+      <c r="C84" s="157"/>
+      <c r="D84" s="157"/>
+      <c r="E84" s="157"/>
+      <c r="F84" s="158"/>
+    </row>
+    <row r="85" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A85" s="159"/>
+      <c r="B85" s="160"/>
+      <c r="C85" s="160"/>
+      <c r="D85" s="160"/>
+      <c r="E85" s="160"/>
+      <c r="F85" s="161"/>
+    </row>
+    <row r="86" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A86" s="159"/>
+      <c r="B86" s="160"/>
+      <c r="C86" s="160"/>
+      <c r="D86" s="160"/>
+      <c r="E86" s="160"/>
+      <c r="F86" s="161"/>
+    </row>
+    <row r="87" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A87" s="159"/>
+      <c r="B87" s="160"/>
+      <c r="C87" s="160"/>
+      <c r="D87" s="160"/>
+      <c r="E87" s="160"/>
+      <c r="F87" s="161"/>
+    </row>
+    <row r="88" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A88" s="159"/>
+      <c r="B88" s="160"/>
+      <c r="C88" s="160"/>
+      <c r="D88" s="160"/>
+      <c r="E88" s="160"/>
+      <c r="F88" s="161"/>
+    </row>
+    <row r="89" spans="1:6" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A89" s="159"/>
+      <c r="B89" s="160"/>
+      <c r="C89" s="160"/>
+      <c r="D89" s="160"/>
+      <c r="E89" s="160"/>
+      <c r="F89" s="161"/>
+    </row>
+    <row r="90" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="159"/>
+      <c r="B90" s="160"/>
+      <c r="C90" s="160"/>
+      <c r="D90" s="160"/>
+      <c r="E90" s="160"/>
+      <c r="F90" s="161"/>
+    </row>
+    <row r="91" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A91" s="159"/>
+      <c r="B91" s="160"/>
+      <c r="C91" s="160"/>
+      <c r="D91" s="160"/>
+      <c r="E91" s="160"/>
+      <c r="F91" s="161"/>
+    </row>
+    <row r="92" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A92" s="159"/>
+      <c r="B92" s="160"/>
+      <c r="C92" s="160"/>
+      <c r="D92" s="160"/>
+      <c r="E92" s="160"/>
+      <c r="F92" s="161"/>
+    </row>
+    <row r="93" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A93" s="159"/>
+      <c r="B93" s="160"/>
+      <c r="C93" s="160"/>
+      <c r="D93" s="160"/>
+      <c r="E93" s="160"/>
+      <c r="F93" s="161"/>
+    </row>
+    <row r="94" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A94" s="159"/>
+      <c r="B94" s="160"/>
+      <c r="C94" s="160"/>
+      <c r="D94" s="160"/>
+      <c r="E94" s="160"/>
+      <c r="F94" s="161"/>
+    </row>
+    <row r="95" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A95" s="159"/>
+      <c r="B95" s="160"/>
+      <c r="C95" s="160"/>
+      <c r="D95" s="160"/>
+      <c r="E95" s="160"/>
+      <c r="F95" s="161"/>
+    </row>
+    <row r="96" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A96" s="159"/>
+      <c r="B96" s="160"/>
+      <c r="C96" s="160"/>
+      <c r="D96" s="160"/>
+      <c r="E96" s="160"/>
+      <c r="F96" s="161"/>
+    </row>
+    <row r="97" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A97" s="159"/>
+      <c r="B97" s="160"/>
+      <c r="C97" s="160"/>
+      <c r="D97" s="160"/>
+      <c r="E97" s="160"/>
+      <c r="F97" s="161"/>
+    </row>
+    <row r="98" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A98" s="159"/>
+      <c r="B98" s="160"/>
+      <c r="C98" s="160"/>
+      <c r="D98" s="160"/>
+      <c r="E98" s="160"/>
+      <c r="F98" s="161"/>
+    </row>
+    <row r="99" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A99" s="159"/>
+      <c r="B99" s="160"/>
+      <c r="C99" s="160"/>
+      <c r="D99" s="160"/>
+      <c r="E99" s="160"/>
+      <c r="F99" s="161"/>
+    </row>
+    <row r="100" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A100" s="159"/>
+      <c r="B100" s="160"/>
+      <c r="C100" s="160"/>
+      <c r="D100" s="160"/>
+      <c r="E100" s="160"/>
+      <c r="F100" s="161"/>
+    </row>
+    <row r="101" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A101" s="159"/>
+      <c r="B101" s="160"/>
+      <c r="C101" s="160"/>
+      <c r="D101" s="160"/>
+      <c r="E101" s="160"/>
+      <c r="F101" s="161"/>
+    </row>
+    <row r="102" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="159"/>
+      <c r="B102" s="160"/>
+      <c r="C102" s="160"/>
+      <c r="D102" s="160"/>
+      <c r="E102" s="160"/>
+      <c r="F102" s="161"/>
+    </row>
+    <row r="103" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A103" s="162"/>
+      <c r="B103" s="163"/>
+      <c r="C103" s="163"/>
+      <c r="D103" s="163"/>
+      <c r="E103" s="163"/>
+      <c r="F103" s="164"/>
     </row>
   </sheetData>
   <mergeCells count="63">
+    <mergeCell ref="A13:F18"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="E8:F8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="E21:E27"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="A28:A33"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="E29:E34"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="A35:A40"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E36:E40"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="A84:F103"/>
+    <mergeCell ref="A56:E56"/>
+    <mergeCell ref="A57:E57"/>
+    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="C59:E59"/>
+    <mergeCell ref="A60:F60"/>
+    <mergeCell ref="A72:F72"/>
     <mergeCell ref="A20:A26"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="A73:F73"/>
@@ -4640,57 +4746,10 @@
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="D43:F43"/>
     <mergeCell ref="D44:F48"/>
-    <mergeCell ref="A84:F103"/>
-    <mergeCell ref="A56:E56"/>
-    <mergeCell ref="A57:E57"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="C59:E59"/>
-    <mergeCell ref="A60:F60"/>
-    <mergeCell ref="A72:F72"/>
     <mergeCell ref="D49:F49"/>
-    <mergeCell ref="A35:A40"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="E36:E40"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="A28:A33"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="E29:E34"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="E21:E27"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="A13:F18"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F3"/>
-    <mergeCell ref="B4:F4"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="E8:F8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="63" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -4703,13 +4762,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>42</xdr:row>
-                    <xdr:rowOff>219075</xdr:rowOff>
+                    <xdr:rowOff>220980</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>66675</xdr:colOff>
+                    <xdr:colOff>68580</xdr:colOff>
                     <xdr:row>44</xdr:row>
                     <xdr:rowOff>38100</xdr:rowOff>
                   </to>
@@ -4725,13 +4784,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>43</xdr:row>
-                    <xdr:rowOff>142875</xdr:rowOff>
+                    <xdr:rowOff>144780</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>45</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4747,15 +4806,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>45</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>66675</xdr:colOff>
+                    <xdr:colOff>68580</xdr:colOff>
                     <xdr:row>47</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4769,13 +4828,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>46</xdr:row>
                     <xdr:rowOff>152400</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>48</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4791,15 +4850,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>47</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>49</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4813,15 +4872,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>48</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>50</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4835,15 +4894,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>49</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>51</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4859,11 +4918,11 @@
                     <xdr:col>1</xdr:col>
                     <xdr:colOff>533400</xdr:colOff>
                     <xdr:row>50</xdr:row>
-                    <xdr:rowOff>161925</xdr:rowOff>
+                    <xdr:rowOff>160020</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>52</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4879,13 +4938,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>51</xdr:row>
                     <xdr:rowOff>152400</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>53</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4901,13 +4960,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>523875</xdr:colOff>
+                    <xdr:colOff>525780</xdr:colOff>
                     <xdr:row>44</xdr:row>
-                    <xdr:rowOff>161925</xdr:rowOff>
+                    <xdr:rowOff>160020</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>66675</xdr:colOff>
+                    <xdr:colOff>68580</xdr:colOff>
                     <xdr:row>46</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4923,13 +4982,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>809625</xdr:colOff>
+                    <xdr:colOff>807720</xdr:colOff>
                     <xdr:row>7</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>971550</xdr:colOff>
+                    <xdr:colOff>975360</xdr:colOff>
                     <xdr:row>8</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -4945,15 +5004,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>857250</xdr:colOff>
+                    <xdr:colOff>861060</xdr:colOff>
                     <xdr:row>6</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>1552575</xdr:colOff>
+                    <xdr:colOff>1554480</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>9525</xdr:rowOff>
+                    <xdr:rowOff>7620</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4967,15 +5026,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>57150</xdr:colOff>
+                    <xdr:colOff>60960</xdr:colOff>
                     <xdr:row>8</xdr:row>
-                    <xdr:rowOff>171450</xdr:rowOff>
+                    <xdr:rowOff>175260</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>1</xdr:col>
-                    <xdr:colOff>219075</xdr:colOff>
+                    <xdr:colOff>220980</xdr:colOff>
                     <xdr:row>9</xdr:row>
-                    <xdr:rowOff>161925</xdr:rowOff>
+                    <xdr:rowOff>160020</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -4991,21 +5050,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K61"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.28515625" style="41" customWidth="1"/>
-    <col min="2" max="2" width="43.7109375" style="22" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" style="22" customWidth="1"/>
-    <col min="4" max="4" width="41.85546875" style="22" customWidth="1"/>
-    <col min="5" max="5" width="34.28515625" style="22" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" style="22" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="22" customWidth="1"/>
-    <col min="8" max="8" width="16.28515625" style="46" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" style="22" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="22"/>
+    <col min="1" max="1" width="6.33203125" style="41" customWidth="1"/>
+    <col min="2" max="2" width="43.6640625" style="22" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" style="22" customWidth="1"/>
+    <col min="4" max="4" width="41.88671875" style="22" customWidth="1"/>
+    <col min="5" max="5" width="34.33203125" style="22" customWidth="1"/>
+    <col min="6" max="6" width="9.88671875" style="22" customWidth="1"/>
+    <col min="7" max="7" width="10.6640625" style="22" customWidth="1"/>
+    <col min="8" max="8" width="16.33203125" style="46" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" style="22" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="22"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="22.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="47" t="s">
         <v>70</v>
       </c>
@@ -5034,7 +5093,7 @@
       <c r="J1" s="20"/>
       <c r="K1" s="21"/>
     </row>
-    <row r="2" spans="1:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="40">
         <v>1</v>
       </c>
@@ -5064,7 +5123,7 @@
       <c r="J2" s="23"/>
       <c r="K2" s="21"/>
     </row>
-    <row r="3" spans="1:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="40">
         <v>2</v>
       </c>
@@ -5094,7 +5153,7 @@
       <c r="J3" s="23"/>
       <c r="K3" s="21"/>
     </row>
-    <row r="4" spans="1:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="40">
         <v>3</v>
       </c>
@@ -5124,7 +5183,7 @@
       <c r="J4" s="23"/>
       <c r="K4" s="21"/>
     </row>
-    <row r="5" spans="1:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="40">
         <v>4</v>
       </c>
@@ -5154,7 +5213,7 @@
       <c r="J5" s="23"/>
       <c r="K5" s="21"/>
     </row>
-    <row r="6" spans="1:11" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="40">
         <v>5</v>
       </c>
@@ -5181,55 +5240,55 @@
         <v>4.25</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D8" s="222" t="s">
+    <row r="8" spans="1:11" ht="15.45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="221" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="222"/>
-      <c r="F8" s="222"/>
-      <c r="G8" s="222"/>
-      <c r="H8" s="223">
+      <c r="E8" s="221"/>
+      <c r="F8" s="221"/>
+      <c r="G8" s="221"/>
+      <c r="H8" s="222">
         <f>SUM(H2:H6)</f>
         <v>50.849999999999994</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="14.65" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D9" s="222"/>
-      <c r="E9" s="222"/>
-      <c r="F9" s="222"/>
-      <c r="G9" s="222"/>
-      <c r="H9" s="223"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="14.7" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D9" s="221"/>
+      <c r="E9" s="221"/>
+      <c r="F9" s="221"/>
+      <c r="G9" s="221"/>
+      <c r="H9" s="222"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B11" s="38"/>
       <c r="C11" s="38"/>
       <c r="E11" s="38"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="B12" s="37"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B13" s="37"/>
     </row>
-    <row r="14" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B14" s="33" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="34" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B16" s="35" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B17" s="37"/>
     </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B18" s="38"/>
       <c r="C18" s="38"/>
       <c r="D18" s="38"/>
@@ -5237,28 +5296,28 @@
       <c r="F18" s="38"/>
       <c r="G18" s="38"/>
     </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B19" s="37"/>
       <c r="C19" s="37"/>
       <c r="E19" s="37"/>
       <c r="F19" s="37"/>
       <c r="G19" s="37"/>
     </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B20" s="37"/>
       <c r="C20" s="37"/>
       <c r="E20" s="37"/>
       <c r="F20" s="37"/>
       <c r="G20" s="37"/>
     </row>
-    <row r="21" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B21" s="37"/>
       <c r="C21" s="37"/>
       <c r="E21" s="37"/>
       <c r="F21" s="37"/>
       <c r="G21" s="37"/>
     </row>
-    <row r="22" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B22" s="37"/>
       <c r="C22" s="37"/>
       <c r="D22"/>
@@ -5266,7 +5325,7 @@
       <c r="F22" s="37"/>
       <c r="G22" s="37"/>
     </row>
-    <row r="23" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B23" s="37"/>
       <c r="C23" s="37"/>
       <c r="D23"/>
@@ -5274,7 +5333,7 @@
       <c r="F23" s="37"/>
       <c r="G23" s="37"/>
     </row>
-    <row r="24" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B24" s="37"/>
       <c r="C24" s="37"/>
       <c r="D24" s="44"/>
@@ -5282,7 +5341,7 @@
       <c r="F24" s="37"/>
       <c r="G24" s="37"/>
     </row>
-    <row r="25" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B25" s="37"/>
       <c r="C25" s="37"/>
       <c r="D25"/>
@@ -5290,7 +5349,7 @@
       <c r="F25" s="37"/>
       <c r="G25" s="37"/>
     </row>
-    <row r="26" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B26" s="37"/>
       <c r="C26" s="37"/>
       <c r="D26"/>
@@ -5298,7 +5357,7 @@
       <c r="F26" s="37"/>
       <c r="G26" s="37"/>
     </row>
-    <row r="27" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B27" s="37"/>
       <c r="C27" s="37"/>
       <c r="D27" s="44"/>
@@ -5306,7 +5365,7 @@
       <c r="F27" s="37"/>
       <c r="G27" s="37"/>
     </row>
-    <row r="28" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B28" s="37"/>
       <c r="C28" s="37"/>
       <c r="D28"/>
@@ -5314,7 +5373,7 @@
       <c r="F28" s="37"/>
       <c r="G28" s="37"/>
     </row>
-    <row r="29" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B29" s="37"/>
       <c r="C29" s="37"/>
       <c r="D29"/>
@@ -5322,35 +5381,35 @@
       <c r="F29" s="37"/>
       <c r="G29" s="37"/>
     </row>
-    <row r="30" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B30" s="37"/>
       <c r="C30" s="37"/>
       <c r="E30" s="37"/>
       <c r="F30" s="37"/>
       <c r="G30" s="37"/>
     </row>
-    <row r="31" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B31" s="37"/>
       <c r="C31" s="37"/>
       <c r="E31" s="37"/>
       <c r="F31" s="37"/>
       <c r="G31" s="37"/>
     </row>
-    <row r="32" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B32" s="37"/>
       <c r="C32" s="37"/>
       <c r="E32" s="37"/>
       <c r="F32" s="37"/>
       <c r="G32" s="37"/>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B33" s="37"/>
       <c r="C33" s="37"/>
       <c r="E33" s="37"/>
       <c r="F33" s="37"/>
       <c r="G33" s="37"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="41">
         <v>1</v>
       </c>
@@ -5358,7 +5417,7 @@
       <c r="F34" s="37"/>
       <c r="G34" s="37"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="41">
         <v>2</v>
       </c>
@@ -5366,7 +5425,7 @@
       <c r="F35" s="37"/>
       <c r="G35" s="37"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="41">
         <v>3</v>
       </c>
@@ -5374,7 +5433,7 @@
       <c r="F36" s="37"/>
       <c r="G36" s="37"/>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="41">
         <v>4</v>
       </c>
@@ -5382,7 +5441,7 @@
       <c r="F37" s="37"/>
       <c r="G37" s="37"/>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="41">
         <v>5</v>
       </c>
@@ -5390,7 +5449,7 @@
       <c r="F38" s="37"/>
       <c r="G38" s="37"/>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="41">
         <v>6</v>
       </c>
@@ -5398,7 +5457,7 @@
       <c r="F39" s="37"/>
       <c r="G39" s="37"/>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="41">
         <v>7</v>
       </c>
@@ -5406,7 +5465,7 @@
       <c r="F40" s="37"/>
       <c r="G40" s="37"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="41">
         <v>8</v>
       </c>
@@ -5414,7 +5473,7 @@
       <c r="F41" s="37"/>
       <c r="G41" s="37"/>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="41">
         <v>9</v>
       </c>
@@ -5422,97 +5481,97 @@
       <c r="F42" s="37"/>
       <c r="G42" s="37"/>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="41">
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="41">
         <v>11</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="41">
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="41">
         <v>13</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="41">
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="41">
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="41">
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="41">
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="41">
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="41">
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A53" s="41">
         <v>20</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="41">
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="41">
         <v>22</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="41">
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="41">
         <v>24</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A58" s="41">
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A59" s="41">
         <v>26</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A60" s="41">
         <v>27</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A61" s="41">
         <v>28</v>
       </c>
@@ -5533,28 +5592,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I3"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="37.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="35.28515625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="19.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="37.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="35.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="19.88671875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="20" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="1"/>
+    <col min="7" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A1" s="224" t="s">
+    <row r="1" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A1" s="223" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="224"/>
-      <c r="C1" s="224"/>
-      <c r="D1" s="224"/>
-      <c r="E1" s="224"/>
-      <c r="F1" s="224"/>
-    </row>
-    <row r="2" spans="1:9" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B1" s="223"/>
+      <c r="C1" s="223"/>
+      <c r="D1" s="223"/>
+      <c r="E1" s="223"/>
+      <c r="F1" s="223"/>
+    </row>
+    <row r="2" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A2" s="53"/>
       <c r="B2" s="53"/>
       <c r="C2" s="53"/>
@@ -5565,7 +5624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A3" s="53"/>
       <c r="B3" s="53"/>
       <c r="C3" s="53"/>

</xml_diff>